<commit_message>
Add nine source-reviewed Wuhan University profiles (770 total)
</commit_message>
<xml_diff>
--- a/site/exports/whu-math-stat.xlsx
+++ b/site/exports/whu-math-stat.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导师'!$A$1:$L$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -675,12 +675,120 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>王六权</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>校区未标注</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>数学与统计学院</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>https://jszy.whu.edu.cn/lqwang/</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>官网个人页明示数学与统计学院归属，未独立核目录或实时人事；教师/教授是来源称谓，不推出聘任或晋升日期。；仅必要职业摘录，非完整原页、完整履历或HTTP实体；未披露的导师、研究方向及课程不补造。；原学习区间与授位年月分开；原学位证及历史法律授位实体未单独核实。；作品均仅官网书目，作者原列保留，不将已列姓名当独立外核完整作者名单或贡献认证。</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>公开个人页（访问与内容时效见来源记录）</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>whu</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>武汉大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>王好武</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>校区未标注</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>数学与统计学院</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>https://jszy.whu.edu.cn/wanghaowu/zh_CN/</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>官网个人页明示数学与统计学院归属，未独立核目录或实时人事；教师/教授是来源称谓，不推出聘任或晋升日期。；仅必要职业摘录，非完整原页、完整履历或HTTP实体；未披露的导师、研究方向及课程不补造。；原学习区间与授位年月分开；原学位证及历史法律授位实体未单独核实。；作品均仅官网书目，未核出版元数据与全文；王好武原文及译文同计一作，with合作者不是完整作者顺序。</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>公开个人页（访问与内容时效见来源记录）</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>whu</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>武汉大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K4"/>
+  <autoFilter ref="A1:K6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -692,7 +800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S18"/>
+  <dimension ref="A1:S23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1906,8 +2014,359 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>王六权</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>理学博士</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>新加坡国立大学</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>2014-08</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>2017-08</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>数学</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>官网条目明确理学博士学位，据此记录来源报告的学位；未独立核原证书或法律授位实体，不声称取得未留存的栏目标题。原学习区间保留，授位年月仍未知，不从学习末期推定。</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr"/>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>https://jszy.whu.edu.cn/lqwang/</t>
+        </is>
+      </c>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>whu</t>
+        </is>
+      </c>
+      <c r="S19" s="2" t="inlineStr">
+        <is>
+          <t>武汉大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>王六权</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>学士</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>浙江大学</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>2010-08</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>2014-06</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>数学与应用数学</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>官网条目明确学士学位，据此记录来源报告的学位；未独立核原证书或法律授位实体，不声称取得未留存的栏目标题。原学习区间保留，授位年月仍未知，不从学习末期推定。</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr"/>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>https://jszy.whu.edu.cn/lqwang/</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>whu</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>武汉大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>王好武</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>理学博士</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>法国里尔大学</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>2015-09</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>2019-07</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>基础数学</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>官网条目明确理学博士学位，据此记录来源报告的学位；未独立核原证书或法律授位实体，不声称取得未留存的栏目标题。原学习区间保留，授位年月仍未知，不从学习末期推定。</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>https://jszy.whu.edu.cn/wanghaowu/zh_CN/</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>whu</t>
+        </is>
+      </c>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>武汉大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>王好武</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>学士</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>武汉大学</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>2011-09</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>2015-06</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>基础数学</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>官网条目明确学士及大学本科毕业，据此记录来源报告的学位；未独立核原证书或法律授位实体，不声称取得未留存的栏目标题。原学习区间保留，授位年月仍未知，不从学习末期推定。</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr"/>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>https://jszy.whu.edu.cn/wanghaowu/zh_CN/</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>whu</t>
+        </is>
+      </c>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>武汉大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>王好武</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>postdoctoral_research</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>博士后</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>德国马普数学所</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>2019-10</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>2021-09</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>博士后为非学位研究经历，不否定本人其他学位。</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr"/>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>https://jszy.whu.edu.cn/wanghaowu/zh_CN/</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>whu</t>
+        </is>
+      </c>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>武汉大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S18"/>
+  <autoFilter ref="A1:S23"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -1926,6 +2385,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2140,7 +2604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2148,7 +2612,7 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="51.8" customWidth="1" min="4" max="4"/>
     <col width="65" customWidth="1" min="5" max="5"/>
-    <col width="37.8" customWidth="1" min="6" max="6"/>
+    <col width="51.8" customWidth="1" min="6" max="6"/>
     <col width="65" customWidth="1" min="7" max="7"/>
     <col width="65" customWidth="1" min="8" max="8"/>
     <col width="65" customWidth="1" min="9" max="9"/>
@@ -2511,8 +2975,216 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>王六权</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Nahm sum identities for Cartan matrices of type Dk</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>https://jszy.whu.edu.cn/lqwang/zh_CN/lwcg/465934/list/index.htm</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文；journal_article_as_official_list</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>https://jszy.whu.edu.cn/lqwang/zh_CN/lwcg/465934/list/index.htm</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>仅官网论文列目，未核出版者或全文；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>仅官网论文列目，未独立核出版者元数据或全文；卷期页码按原样保留，不根据作者顺序推贡献角色。</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>whu</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>武汉大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>王六权</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Counterexamples to some duality principles of modular Nahm sums</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>https://jszy.whu.edu.cn/lqwang/zh_CN/lwcg/465934/list/index.htm</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文；journal_article_as_official_list</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>https://jszy.whu.edu.cn/lqwang/zh_CN/lwcg/465934/list/index.htm</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>仅官网论文列目，未核出版者或全文；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>仅官网论文列目，未独立核出版者元数据或全文；卷期页码按原样保留，不根据作者顺序推贡献角色。</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>whu</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>武汉大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>王好武</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Conjecture on first-order theta-blocks</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>https://jszy.whu.edu.cn/wanghaowu/zh_CN/zdylm/1510076/list/index.htm</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文；journal_article_as_official_list</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>https://jszy.whu.edu.cn/wanghaowu/zh_CN/zdylm/1510076/list/index.htm</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>仅官网论文列目，未核出版者或全文；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>仅官网论文列目，未独立核出版者元数据或全文；卷期页码按原样保留，不根据作者顺序推贡献角色。 原列 with V. Gritsenko 为合作者信息，不是完整作者名单或顺序，不能据此认定唯一共同作者。 原文为俄文；译文载 Russian Math. Surveys 72:5 (2017), 968--970，与 Uspekhi Mat. Nauk 72:5(437) (2017), 191-192 同一作品，不增第二篇作品。</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>whu</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>武汉大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>王好武</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Powers of Jacobi triple product, Cohen’s numbers and the Ramanujan \Delta-function</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>2018</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>https://jszy.whu.edu.cn/wanghaowu/zh_CN/zdylm/1510076/list/index.htm</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>期刊论文；journal_article_as_official_list</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>https://jszy.whu.edu.cn/wanghaowu/zh_CN/zdylm/1510076/list/index.htm</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>仅官网论文列目，未核出版者或全文；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>仅官网论文列目，未独立核出版者元数据或全文；卷期页码按原样保留，不根据作者顺序推贡献角色。 原列 with V. Gritsenko 为合作者信息，不是完整作者名单或顺序，不能据此认定唯一共同作者。</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>whu</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>武汉大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L6"/>
+  <autoFilter ref="A1:L10"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
@@ -2529,6 +3201,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2540,7 +3220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3110,27 +3790,27 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>敖微微</t>
+          <t>王六权</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>institution-classification-5</t>
+          <t>whu-wangliuquan-profile</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</t>
+          <t>https://jszy.whu.edu.cn/lqwang/</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>历史985院校分类参考；非个人授位或就读当年建设身份的证明</t>
+          <t>既有必要职业摘录，保留空白归一化与省略原序号说明；非完整原页或HTTP实体；retained_professional_excerpts_checked</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>未单独记录</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -3147,42 +3827,190 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>王六权</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>whu-wangliuquan-works</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>https://jszy.whu.edu.cn/lqwang/zh_CN/lwcg/465934/list/index.htm</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>既有必要职业摘录，保留空白归一化与省略原序号说明；非完整原页或HTTP实体；retained_professional_excerpts_checked</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>whu</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>武汉大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>王好武</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>whu-wanghaowu-profile</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>https://jszy.whu.edu.cn/wanghaowu/zh_CN/</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>既有必要职业摘录，保留空白归一化与省略原序号说明；非完整原页或HTTP实体；retained_professional_excerpts_checked</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>whu</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>武汉大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>王好武</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>whu-wanghaowu-works</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>https://jszy.whu.edu.cn/wanghaowu/zh_CN/zdylm/1510076/list/index.htm</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>既有必要职业摘录，保留空白归一化与省略原序号说明；非完整原页或HTTP实体；retained_professional_excerpts_checked</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>whu</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>武汉大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>敖微微</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>institution-classification-5</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>历史985院校分类参考；非个人授位或就读当年建设身份的证明</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>未单独记录</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>whu</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>武汉大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>陈国贤</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>institution-classification-6</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>历史985院校分类参考；非个人授位或就读当年建设身份的证明</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>未单独记录</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>whu</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>whu</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>武汉大学</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G17"/>
+  <autoFilter ref="A1:G21"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -3200,6 +4028,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>